<commit_message>
Move LNG Canada Phase 2 to the committed scenario after its final investment decision (29 Sep 2026)
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Asset_Register.xlsx
+++ b/Inputs/Canada_LNG_Asset_Register.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset Register" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset Sources" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supporting Infrastructure" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Definitions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Gaps" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Asset Register" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Asset Sources" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Supporting Infrastructure" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Field Definitions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Data Gaps" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Asset Register'!$A$1:$BB$56</definedName>
@@ -27,7 +27,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <name val="Calibri"/>
@@ -111,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -128,6 +130,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -972,7 +975,7 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>It carries 21.46 bcm/y and already serves 24.50 from LNG Canada Phase 1 plus Cedar (3.75 mtpa since the July 2026 certificate amendment), whose 8 km connector draws on it. Phase 2's 14 mtpa, 31 per cent of live export capacity, depends on the proposed second line agreed only in principle in March 2026.</t>
+          <t>It carries 21.46 bcm/y and already serves 24.50 from LNG Canada Phase 1 plus Cedar (3.75 mtpa since the July 2026 certificate amendment), whose 8 km connector draws on it. Phase 2's 14 mtpa depends on the Coastal GasLink expansion, which will proceed following the LNG Canada Phase 2 final investment decision of 29 September 2026.</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1027,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
@@ -1052,7 +1054,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>No FID yet. Status text refreshed; first LNG 2030 reconfirmed (GEM wiki, 25 Sep 2026: https://www.gem.wiki/LNG_Canada_Terminal).</t>
+          <t>Final investment decision 29 Sep 2026. Status construction, tier and calc_group under_construction, first LNG 2031 (decision date plus the IEA 4 to 5 year lag; Shell expects commercial operations in the early 2030s).</t>
         </is>
       </c>
     </row>
@@ -3325,17 +3327,17 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>advanced_proposed</t>
+          <t>under_construction</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>under_construction</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Referred to the Major Projects Office Sep 2025 and designated national interest. Canada, British Columbia and LNG Canada agreed enhanced investment co-operation on 14 May 2026, targeting a 2026 FID. LNG Canada issued a limited notice to proceed to the JGC-Fluor joint venture in June 2026. Reuters reported on 24 Sep 2026 that an FID could come as early as October, and LNG Canada hopes to decide before the end of 2026. No FID as of 27 Sep 2026, so the tier stays advanced_proposed.</t>
+          <t>Final investment decision taken 29 September 2026 by the LNG Canada joint venture (Shell, PETRONAS, PetroChina, Mitsubishi, KOGAS); Fluor joint venture selected for engineering, procurement and construction. Moved from advanced_proposed.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -3360,19 +3362,22 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>construction</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="N11" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="O11" s="12" t="n">
+        <v>46294</v>
       </c>
       <c r="P11" t="n">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="Q11" s="4" t="inlineStr">
         <is>
@@ -3415,7 +3420,11 @@
         <v>3800</v>
       </c>
       <c r="AC11" s="4" t="inlineStr"/>
-      <c r="AE11" s="4" t="inlineStr"/>
+      <c r="AE11" s="4" t="inlineStr">
+        <is>
+          <t>FID 29 Sep 2026; phase 2 cost reported at US$21–23bn (Mitsubishi share US$3.2bn implies US$21.3bn); total terminal capacity 28 mtpa; commercial operation expected in the early 2030s.</t>
+        </is>
+      </c>
       <c r="AF11" t="inlineStr">
         <is>
           <t>export</t>
@@ -3510,7 +3519,7 @@
       </c>
       <c r="BB11" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | NRCan Canadian LNG projects: https://natural-resources.canada.ca/energy-sources/fossil-fuels/canadian-liquified-natural-gas-projects | Major Projects Office, LNG Canada Phase 2: https://www.canada.ca/en/privy-council/major-projects-office/projects/national/lng-canada.html | CER Market Snapshot, Canada's future in LNG exports: https://www.cer-rec.gc.ca/en/data-analysis/energy-markets/market-snapshots/2024/market-snapshot-exploring-canadas-future-in-lng-exports.html | Norton Rose Fulbright, Canadian LNG industry 2026 outlook: https://www.nortonrosefulbright.com/en/knowledge/publications/10bef30f/canadian-lng-industry-2026-outlook | GEM wiki: https://www.gem.wiki/LNG_Canada_Terminal | The Northern View, Phase 2 decision could come as early as October (24 Sep 2026): https://thenorthernview.com/2026/09/24/lng-canada-phase-2-decision-could-come-as-early-as-october/</t>
+          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | NRCan Canadian LNG projects: https://natural-resources.canada.ca/energy-sources/fossil-fuels/canadian-liquified-natural-gas-projects | Major Projects Office, LNG Canada Phase 2: https://www.canada.ca/en/privy-council/major-projects-office/projects/national/lng-canada.html | CER Market Snapshot, Canada's future in LNG exports: https://www.cer-rec.gc.ca/en/data-analysis/energy-markets/market-snapshots/2024/market-snapshot-exploring-canadas-future-in-lng-exports.html | Norton Rose Fulbright, Canadian LNG industry 2026 outlook: https://www.nortonrosefulbright.com/en/knowledge/publications/10bef30f/canadian-lng-industry-2026-outlook | GEM wiki: https://www.gem.wiki/LNG_Canada_Terminal | The Northern View, Phase 2 decision could come as early as October (24 Sep 2026): https://thenorthernview.com/2026/09/24/lng-canada-phase-2-decision-could-come-as-early-as-october/ | LNG Canada, LNG Canada Announces Phase 2 Final Investment Decision (Sep 2026): https://www.newswire.ca/news-releases/lng-canada-announces-phase-2-final-investment-decision-828313121.html | Shell, Shell takes final investment decision on LNG Canada Phase 2 (29 Sep 2026): https://news.europawire.eu/shell-takes-final-investment-decision-on-lng-canada-phase-2-to-double-kitimat-production-capacity-to-28-million-tonnes-per-year/eu-press-release/2026/09/29/14/54/00/181489/ | Financial Times, Shell-led consortium backs $23bn expansion of LNG Canada project (29 Sep 2026): https://www.ft.com/content/364d5454-876d-42ef-8f30-759e1ebdb026 | Fluor, Fluor joint venture selected for LNG Canada Phase 2 expansion following final investment decision (29 Sep 2026): https://www.financialcontent.com/article/bizwire-2026-9-29-fluor-joint-venture-selected-for-lng-canada-phase-2-expansion-following-final-investment-decision | TC Energy, Coastal GasLink Phase 2 to proceed following LNG Canada Final Investment Decision (29 Sep 2026): https://www.globenewswire.com/news-release/2026/09/29/3370625/0/en/coastal-gaslink-phase-2-to-proceed-following-lng-canada-final-investment-decision.html</t>
         </is>
       </c>
       <c r="BC11" t="inlineStr">
@@ -13081,17 +13090,17 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Assigned by us from status, regulatory stage and FID - see tier_reason</t>
+          <t>Moved from advanced_proposed after the 29 Sep 2026 final investment decision. LNG Canada, LNG Canada Announces Phase 2 Final Investment Decision (Sep 2026): https://www.newswire.ca/news-releases/lng-canada-announces-phase-2-final-investment-decision-828313121.html</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Derived: advanced_proposed and early_proposed group as proposed</t>
+          <t>Follows tier after the 29 Sep 2026 final investment decision. Committed is operating plus under_construction.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Major Projects Office, LNG Canada Phase 2 (modified 2 Jul 2026): https://www.canada.ca/en/privy-council/major-projects-office/projects/national/lng-canada.html | GEM wiki, LNG Canada Terminal (edited 25 Sep 2026): https://www.gem.wiki/LNG_Canada_Terminal | The Northern View, 24 Sep 2026 (Reuters): https://thenorthernview.com/2026/09/24/lng-canada-phase-2-decision-could-come-as-early-as-october/</t>
+          <t>Final investment decision taken 29 September 2026 by the LNG Canada joint venture (Shell, PETRONAS, PetroChina, Mitsubishi, KOGAS); Fluor joint venture selected for engineering, procurement and construction. Moved from advanced_proposed. LNG Canada, LNG Canada Announces Phase 2 Final Investment Decision (Sep 2026): https://www.newswire.ca/news-releases/lng-canada-announces-phase-2-final-investment-decision-828313121.html | Shell, Shell takes final investment decision on LNG Canada Phase 2 (29 Sep 2026): https://news.europawire.eu/shell-takes-final-investment-decision-on-lng-canada-phase-2-to-double-kitimat-production-capacity-to-28-million-tonnes-per-year/eu-press-release/2026/09/29/14/54/00/181489/ | Financial Times, Shell-led consortium backs $23bn expansion of LNG Canada project (29 Sep 2026): https://www.ft.com/content/364d5454-876d-42ef-8f30-759e1ebdb026 | Fluor, Fluor joint venture selected for LNG Canada Phase 2 expansion following final investment decision (29 Sep 2026): https://www.financialcontent.com/article/bizwire-2026-9-29-fluor-joint-venture-selected-for-lng-canada-phase-2-expansion-following-final-investment-decision | TC Energy, Coastal GasLink Phase 2 to proceed following LNG Canada Final Investment Decision (29 Sep 2026): https://www.globenewswire.com/news-release/2026/09/29/3370625/0/en/coastal-gaslink-phase-2-to-proceed-following-lng-canada-final-investment-decision.html</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -13116,7 +13125,7 @@
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ (proposed); Major Projects Office, LNG Canada Phase 2: https://www.canada.ca/en/privy-council/major-projects-office/projects/national/lng-canada.html</t>
+          <t>Post-FID value used by Cedar LNG and Woodfibre LNG. Field Definitions: GEM status vocabulary operating, construction, proposed, shelved, cancelled. LNG Canada, LNG Canada Announces Phase 2 Final Investment Decision (Sep 2026): https://www.newswire.ca/news-releases/lng-canada-announces-phase-2-final-investment-decision-828313121.html</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
@@ -13126,17 +13135,17 @@
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ FIDStatus=Pre-FID; FID targeted 2026 per Major Projects Office, LNG Canada Phase 2: https://www.canada.ca/en/privy-council/major-projects-office/projects/national/lng-canada.html</t>
+          <t>Final investment decision 29 Sep 2026. LNG Canada, LNG Canada Announces Phase 2 Final Investment Decision (Sep 2026): https://www.newswire.ca/news-releases/lng-canada-announces-phase-2-final-investment-decision-828313121.html | Shell, Shell takes final investment decision on LNG Canada Phase 2 (29 Sep 2026): https://news.europawire.eu/shell-takes-final-investment-decision-on-lng-canada-phase-2-to-double-kitimat-production-capacity-to-28-million-tonnes-per-year/eu-press-release/2026/09/29/14/54/00/181489/</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Announced 28 September 2026 Pacific time, 29 September 2026 UK time. LNG Canada, LNG Canada Announces Phase 2 Final Investment Decision (Sep 2026): https://www.newswire.ca/news-releases/lng-canada-announces-phase-2-final-investment-decision-828313121.html | Shell, Shell takes final investment decision on LNG Canada Phase 2 (29 Sep 2026): https://news.europawire.eu/shell-takes-final-investment-decision-on-lng-canada-phase-2-to-double-kitimat-production-capacity-to-28-million-tonnes-per-year/eu-press-release/2026/09/29/14/54/00/181489/</t>
         </is>
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>GEM wiki, LNG Canada Terminal (edited 25 Sep 2026): https://www.gem.wiki/LNG_Canada_Terminal - planned first LNG for Phase 2 is 2030. Unchanged from GEM GGIT (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ LatestPlannedStartYear=2030. No developer date published; replace with the date given at FID.</t>
+          <t>2031: decision date September 2026 plus the IEA's 4 to 5 year lag from final investment decision to completion (Parameters post_fid_to_completion = 4.5), consistent with Shell's statement that commercial operations are expected in the early 2030s. Decision 29 Sep 2026. Shell, Shell takes final investment decision on LNG Canada Phase 2 (29 Sep 2026): https://news.europawire.eu/shell-takes-final-investment-decision-on-lng-canada-phase-2-to-double-kitimat-production-capacity-to-28-million-tonnes-per-year/eu-press-release/2026/09/29/14/54/00/181489/</t>
         </is>
       </c>
       <c r="Q11" s="4" t="inlineStr">
@@ -13211,7 +13220,7 @@
       </c>
       <c r="AE11" s="4" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>FID 29 Sep 2026; phase 2 cost reported at US$21–23bn (Mitsubishi share US$3.2bn implies US$21.3bn); total terminal capacity 28 mtpa; commercial operation expected in the early 2030s. LNG Canada, LNG Canada Announces Phase 2 Final Investment Decision (Sep 2026): https://www.newswire.ca/news-releases/lng-canada-announces-phase-2-final-investment-decision-828313121.html | Shell, Shell takes final investment decision on LNG Canada Phase 2 (29 Sep 2026): https://news.europawire.eu/shell-takes-final-investment-decision-on-lng-canada-phase-2-to-double-kitimat-production-capacity-to-28-million-tonnes-per-year/eu-press-release/2026/09/29/14/54/00/181489/ | Financial Times, Shell-led consortium backs $23bn expansion of LNG Canada project (29 Sep 2026): https://www.ft.com/content/364d5454-876d-42ef-8f30-759e1ebdb026</t>
         </is>
       </c>
       <c r="AF11" s="4" t="inlineStr">
@@ -28445,12 +28454,12 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>The single largest piece of new gas infrastructure proposed in Canada. LNG Canada and the Coastal GasLink owners agreed in March 2026 to cooperate on expanding capacity. Phase 2 cannot physically run without it.</t>
+          <t>The single largest piece of new gas infrastructure proposed in Canada. LNG Canada and the Coastal GasLink owners agreed in March 2026 to cooperate on expanding capacity. Phase 2 cannot physically run without it. Phase 2 expansion to proceed following the LNG Canada Phase 2 FID (29 Sep 2026)</t>
         </is>
       </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT Gas Pipelines (Nov 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/</t>
+          <t>GEM GGIT Gas Pipelines (Nov 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | TC Energy, Coastal GasLink Phase 2 to proceed following LNG Canada Final Investment Decision (29 Sep 2026): https://www.globenewswire.com/news-release/2026/09/29/3370625/0/en/coastal-gaslink-phase-2-to-proceed-following-lng-canada-final-investment-decision.html</t>
         </is>
       </c>
     </row>

</xml_diff>